<commit_message>
fix(sycebnl-notes): remplissage Notes 13,16,17B,24,26,27,29A,31 depuis balance Trois Soeurs 2024 + correction NOTE26 (retrait lignes hors-perimetre) + fullCalcOnLoad
</commit_message>
<xml_diff>
--- a/backups/EF_SYSCEBNL_Juin (1).xlsx
+++ b/backups/EF_SYSCEBNL_Juin (1).xlsx
@@ -115,7 +115,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="51">'CORRESPONDANCE-BILAN'!$A1:$H41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="52">'CORRESPONDANCE-RESULTAT'!$A1:$E36</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr fullCalcOnLoad="1" calcId="171027"/>
 </workbook>
 </file>
 
@@ -14406,7 +14406,7 @@
         <v>695</v>
       </c>
       <c r="B8" s="169">
-        <v>98375375</v>
+        <v>2417077</v>
       </c>
       <c r="C8" s="169">
         <v>86376516</v>
@@ -14544,7 +14544,9 @@
       <c r="A17" s="169" t="s">
         <v>704</v>
       </c>
-      <c r="B17" s="169"/>
+      <c r="B17" s="169">
+        <v>374029</v>
+      </c>
       <c r="C17" s="169"/>
       <c r="D17" s="169">
         <f t="shared" si="0"/>
@@ -15165,7 +15167,7 @@
         <v>729</v>
       </c>
       <c r="B11" s="169">
-        <v>87805922</v>
+        <v>2048134</v>
       </c>
       <c r="C11" s="169">
         <v>55859517</v>
@@ -16096,9 +16098,9 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
   <dimension ref="A6:F27"/>
-  <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.44140625" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="0.25" defaultColWidth="11.44140625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.77734375" style="133" customWidth="1"/>
     <col min="2" max="2" width="8.77734375" style="133" customWidth="1"/>
@@ -16107,7 +16109,7 @@
     <col min="5" max="16384" width="11.44140625" style="133" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" ns2:dyDescent="0.25">
       <c r="A6" s="327" t="s">
         <v>399</v>
       </c>
@@ -16125,7 +16127,7 @@
       </c>
       <c r="F6" s="336"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ns2:dyDescent="0.25">
       <c r="A7" s="331"/>
       <c r="B7" s="331"/>
       <c r="C7" s="331"/>
@@ -16137,7 +16139,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ns2:dyDescent="0.25">
       <c r="A8" s="169" t="s">
         <v>748</v>
       </c>
@@ -16157,13 +16159,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="27.6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" ht="27.6" customHeight="1" spans="1:6" ns2:dyDescent="0.25">
       <c r="A9" s="174" t="s">
         <v>749</v>
       </c>
-      <c r="B9" s="169"/>
+      <c r="B9" s="169">
+        <v>0</v>
+      </c>
       <c r="C9" s="169">
-        <v>0</v>
+        <v>21668078</v>
       </c>
       <c r="D9" s="169">
         <v>0</v>
@@ -16177,7 +16181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" ns2:dyDescent="0.25">
       <c r="A10" s="169" t="s">
         <v>750</v>
       </c>
@@ -16197,7 +16201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ns2:dyDescent="0.25">
       <c r="A11" s="169" t="s">
         <v>751</v>
       </c>
@@ -16217,7 +16221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" ns2:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>752</v>
       </c>
@@ -16239,7 +16243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="27.6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" ht="27.6" customHeight="1" spans="1:6" ns2:dyDescent="0.25">
       <c r="A13" s="174" t="s">
         <v>753</v>
       </c>
@@ -16259,7 +16263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ns2:dyDescent="0.25">
       <c r="A14" s="169" t="s">
         <v>754</v>
       </c>
@@ -16279,7 +16283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ns2:dyDescent="0.25">
       <c r="A15" s="169" t="s">
         <v>755</v>
       </c>
@@ -16299,7 +16303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ns2:dyDescent="0.25">
       <c r="A16" s="181" t="s">
         <v>756</v>
       </c>
@@ -16321,7 +16325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ns2:dyDescent="0.25">
       <c r="A17" s="418" t="s">
         <v>102</v>
       </c>
@@ -16343,7 +16347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="14.4" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" ht="14.4" customHeight="1" spans="1:6" ns2:dyDescent="0.25">
       <c r="A19" s="419" t="s">
         <v>444</v>
       </c>
@@ -16353,7 +16357,7 @@
       <c r="E19" s="300"/>
       <c r="F19" s="300"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ns2:dyDescent="0.25">
       <c r="A20" s="300" t="s">
         <v>757</v>
       </c>
@@ -16363,7 +16367,7 @@
       <c r="E20" s="300"/>
       <c r="F20" s="300"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" ns2:dyDescent="0.25">
       <c r="A21" s="300" t="s">
         <v>758</v>
       </c>
@@ -16373,7 +16377,7 @@
       <c r="E21" s="300"/>
       <c r="F21" s="300"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ns2:dyDescent="0.25">
       <c r="A22" s="300" t="s">
         <v>759</v>
       </c>
@@ -16383,7 +16387,7 @@
       <c r="E22" s="300"/>
       <c r="F22" s="300"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" ns2:dyDescent="0.25">
       <c r="A23" s="300" t="s">
         <v>760</v>
       </c>
@@ -16393,7 +16397,7 @@
       <c r="E23" s="300"/>
       <c r="F23" s="300"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" ns2:dyDescent="0.25">
       <c r="A24" s="300" t="s">
         <v>761</v>
       </c>
@@ -16403,7 +16407,7 @@
       <c r="E24" s="300"/>
       <c r="F24" s="300"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" ns2:dyDescent="0.25">
       <c r="A25" s="300" t="s">
         <v>762</v>
       </c>
@@ -16413,7 +16417,7 @@
       <c r="E25" s="300"/>
       <c r="F25" s="300"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ns2:dyDescent="0.25">
       <c r="A26" s="300" t="s">
         <v>763</v>
       </c>
@@ -16423,7 +16427,7 @@
       <c r="E26" s="300"/>
       <c r="F26" s="300"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ns2:dyDescent="0.25">
       <c r="A27" s="300" t="s">
         <v>764</v>
       </c>
@@ -19257,7 +19261,7 @@
         <v>886</v>
       </c>
       <c r="B21" s="169">
-        <v>0</v>
+        <v>89268</v>
       </c>
       <c r="C21" s="169">
         <v>0</v>
@@ -20315,9 +20319,9 @@
 </file>
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac">
   <dimension ref="A6:E31"/>
-  <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="11.44140625" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="0" outlineLevelCol="0" ns2:dyDescent="0.25" defaultColWidth="11.44140625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="45.5546875" style="133" customWidth="1"/>
     <col min="2" max="3" width="11.44140625" style="133" customWidth="1"/>
@@ -20326,7 +20330,7 @@
     <col min="6" max="16384" width="11.44140625" style="133" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ns2:dyDescent="0.25">
       <c r="A6" s="337" t="s">
         <v>399</v>
       </c>
@@ -20341,7 +20345,7 @@
       </c>
       <c r="E6" s="341"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ns2:dyDescent="0.25">
       <c r="A7" s="337"/>
       <c r="B7" s="341"/>
       <c r="C7" s="341"/>
@@ -20352,7 +20356,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ns2:dyDescent="0.25">
       <c r="A8" s="174" t="s">
         <v>907</v>
       </c>
@@ -20371,12 +20375,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ns2:dyDescent="0.25">
       <c r="A9" s="174" t="s">
         <v>908</v>
       </c>
       <c r="B9" s="169">
-        <v>450000</v>
+        <v>516000</v>
       </c>
       <c r="C9" s="169">
         <v>17767356</v>
@@ -20390,7 +20394,7 @@
         <v>-97.46726524756976</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ns2:dyDescent="0.25">
       <c r="A10" s="174" t="s">
         <v>909</v>
       </c>
@@ -20409,7 +20413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ns2:dyDescent="0.25">
       <c r="A11" s="174" t="s">
         <v>910</v>
       </c>
@@ -20428,7 +20432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ns2:dyDescent="0.25">
       <c r="A12" s="174" t="s">
         <v>911</v>
       </c>
@@ -20447,7 +20451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ns2:dyDescent="0.25">
       <c r="A13" s="174" t="s">
         <v>912</v>
       </c>
@@ -20466,12 +20470,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ns2:dyDescent="0.25">
       <c r="A14" s="174" t="s">
         <v>913</v>
       </c>
       <c r="B14" s="169">
-        <v>710000</v>
+        <v>0</v>
       </c>
       <c r="C14" s="169">
         <v>8533784</v>
@@ -20485,12 +20489,12 @@
         <v>-91.68012689329845</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ns2:dyDescent="0.25">
       <c r="A15" s="174" t="s">
         <v>914</v>
       </c>
       <c r="B15" s="169">
-        <v>0</v>
+        <v>2550000</v>
       </c>
       <c r="C15" s="169">
         <v>0</v>
@@ -20504,12 +20508,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ns2:dyDescent="0.25">
       <c r="A16" s="174" t="s">
         <v>915</v>
       </c>
       <c r="B16" s="169">
-        <v>264623</v>
+        <v>7300</v>
       </c>
       <c r="C16" s="169">
         <v>108478</v>
@@ -20523,12 +20527,12 @@
         <v>143.9416287173436</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ns2:dyDescent="0.25">
       <c r="A17" s="174" t="s">
         <v>916</v>
       </c>
       <c r="B17" s="169">
-        <v>33651899</v>
+        <v>450000</v>
       </c>
       <c r="C17" s="169">
         <v>4826500</v>
@@ -20542,12 +20546,12 @@
         <v>597.2319278980627</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ns2:dyDescent="0.25">
       <c r="A18" s="174" t="s">
         <v>917</v>
       </c>
       <c r="B18" s="169">
-        <v>0</v>
+        <v>145000</v>
       </c>
       <c r="C18" s="169">
         <v>0</v>
@@ -20561,12 +20565,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="27.6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" ht="27.6" customHeight="1" spans="1:5" ns2:dyDescent="0.25">
       <c r="A19" s="174" t="s">
         <v>918</v>
       </c>
       <c r="B19" s="169">
-        <v>165001</v>
+        <v>0</v>
       </c>
       <c r="C19" s="169">
         <v>0</v>
@@ -20580,7 +20584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ns2:dyDescent="0.25">
       <c r="A20" s="174" t="s">
         <v>919</v>
       </c>
@@ -20599,7 +20603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ns2:dyDescent="0.25">
       <c r="A21" s="174" t="s">
         <v>920</v>
       </c>
@@ -20618,7 +20622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ns2:dyDescent="0.25">
       <c r="A22" s="174" t="s">
         <v>921</v>
       </c>
@@ -20637,12 +20641,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" ns2:dyDescent="0.25">
       <c r="A23" s="174" t="s">
         <v>922</v>
       </c>
       <c r="B23" s="169">
-        <v>0</v>
+        <v>1298000</v>
       </c>
       <c r="C23" s="169">
         <v>22817000</v>
@@ -20656,9 +20660,15 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="174"/>
-      <c r="B24" s="169"/>
+    <row r="24" spans="1:5" ns2:dyDescent="0.25">
+      <c r="A24" s="174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Réception</t>
+        </is>
+      </c>
+      <c r="B24" s="169">
+        <v>1553000</v>
+      </c>
       <c r="C24" s="169"/>
       <c r="D24" s="169">
         <f t="shared" si="0"/>
@@ -20669,7 +20679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" ns2:dyDescent="0.25">
       <c r="A25" s="209" t="s">
         <v>435</v>
       </c>
@@ -20690,16 +20700,16 @@
         <v>-34.80205341715902</v>
       </c>
     </row>
-    <row r="27" ht="14.4" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" ht="14.4" customHeight="1" spans="1:2" ns2:dyDescent="0.25">
       <c r="A27" s="411" t="s">
         <v>471</v>
       </c>
       <c r="B27" s="442"/>
     </row>
-    <row r="28" ht="1.2" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" ht="1.2" customHeight="1" spans="1:1" ns2:dyDescent="0.25">
       <c r="A28" s="443"/>
     </row>
-    <row r="29" ht="35.7" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" ht="35.7" customHeight="1" spans="1:5" ns2:dyDescent="0.25">
       <c r="A29" s="444" t="s">
         <v>923</v>
       </c>
@@ -20708,12 +20718,12 @@
       <c r="D29" s="444"/>
       <c r="E29" s="444"/>
     </row>
-    <row r="30" ht="14.4" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" ht="14.4" customHeight="1" spans="1:3" ns2:dyDescent="0.25">
       <c r="A30" s="445"/>
       <c r="B30" s="445"/>
       <c r="C30" s="445"/>
     </row>
-    <row r="31" ht="14.4" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" ht="14.4" customHeight="1" spans="1:1" ns2:dyDescent="0.25">
       <c r="A31" s="443"/>
     </row>
   </sheetData>
@@ -20770,7 +20780,7 @@
         <v>924</v>
       </c>
       <c r="B8" s="454">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="C8" s="454">
         <v>0</v>
@@ -21249,7 +21259,7 @@
         <v>942</v>
       </c>
       <c r="B8" s="463">
-        <v>0</v>
+        <v>6685920</v>
       </c>
       <c r="C8" s="463">
         <v>0</v>
@@ -21268,7 +21278,7 @@
         <v>943</v>
       </c>
       <c r="B9" s="464">
-        <v>0</v>
+        <v>6965000</v>
       </c>
       <c r="C9" s="169">
         <v>0</v>
@@ -21306,7 +21316,7 @@
         <v>945</v>
       </c>
       <c r="B11" s="464">
-        <v>0</v>
+        <v>669246</v>
       </c>
       <c r="C11" s="169">
         <v>0</v>
@@ -23156,7 +23166,7 @@
         <v>1032</v>
       </c>
       <c r="B17" s="169">
-        <v>0</v>
+        <v>4268</v>
       </c>
       <c r="C17" s="169">
         <v>0</v>

</xml_diff>